<commit_message>
Carga de nuevos trabajos
</commit_message>
<xml_diff>
--- a/resumen_trabajos_1.xlsx
+++ b/resumen_trabajos_1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dacm/we/odoo_con_trabajos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA42FCF1-A245-1D4E-BC71-CC4960E3C1BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1CE5DB7-6E26-FA46-9496-21549D460ACA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="36220" yWindow="-4820" windowWidth="33600" windowHeight="19320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4180" yWindow="600" windowWidth="29420" windowHeight="19320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="430" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="434" uniqueCount="197">
   <si>
     <t>OT</t>
   </si>
@@ -103,60 +103,7 @@
 Pozo aún se encuentra en periodo de mantenimiento.</t>
   </si>
   <si>
-    <t>Matías Pomar</t>
-  </si>
-  <si>
-    <t>Levantamiento tecnico nuevo punto</t>
-  </si>
-  <si>
-    <t>Farellones</t>
-  </si>
-  <si>
-    <t>[Farellones] Planta de Tratamiento</t>
-  </si>
-  <si>
-    <t>LT</t>
-  </si>
-  <si>
-    <t>26/11/2025</t>
-  </si>
-  <si>
-    <t>Felipe Brain</t>
-  </si>
-  <si>
-    <t>Alcance:
-El cliente realizará una intervención en la línea de aducción para habilitar una bifurcación destinada al llenado del tranque. En este punto se instalarán dos válvulas ON/OFF para el control del flujo y un caudalímetro Siemens MAG 5100W para medir el caudal que alimentará el tranque.
-El cliente también informó que construirá una cámara enterrada con tapa, donde quedará instalado el conjunto de válvulas y el caudalímetro. Además, mencionó que puede realizar la instalación mecánica de los equipos, por lo que nosotros debemos considerar la supervisión del montaje y la entrega de planos de canalización. La modificación de la tubería será en HDPE, y es necesario contemplar los anillos del caudalímetro para su correcta instalación. 
-Adicionalmente, se incorporará un switch de comunicaciones que será instalado en la Planta de Tratamiento de Farellones para integrar los equipos LoRa. También se deben considerar los cables y suministros necesarios para el conexionado de los equipos.</t>
-  </si>
-  <si>
     <t>Elías Sanchez</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mantenimiento preventivo </t>
-  </si>
-  <si>
-    <t>[Gestión Hídrica El Soldado] Pozo El Melón N° 04 (PEM-04) Nodo A11</t>
-  </si>
-  <si>
-    <t>05/12/2025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Superintendencia de recursos hidricos </t>
-  </si>
-  <si>
-    <t xml:space="preserve">43 mts esta instalado el sensor hidrostatico 
-Y el pozometro sonó a los 4,10m. 
-Se realiza limpieza al flowcell de la sonda multiparamétrica en el punto. 
-Se anota en Excel interno volumen, Caudal, número de sensor, rango, se revisa programación para corroborar que esta actualizando los datos en el plc. </t>
-  </si>
-  <si>
-    <t>[Gestión Hídrica El Soldado] Pozo El Melón N° 10 (PEM-10) Nodo A16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6,16m suena el pozometro
-Se ajusta el sensor hidrostatico a nivel 0 de la superficie, se corrige el total en metros a través de la transformación de presión bar
-Limpieza, reapriete, verificación de programas ecostruxture, que actualice los datos de sonda y de caudal(en funcionamiento) se actualiza  el volumen,limpieza de flowcell. </t>
   </si>
   <si>
     <t xml:space="preserve">Transporte de materiales </t>
@@ -192,6 +139,9 @@
   </si>
   <si>
     <t>Recinto PME-09, P6 Dren Muro Este</t>
+  </si>
+  <si>
+    <t>LT</t>
   </si>
   <si>
     <t xml:space="preserve">Patricio Cortes </t>
@@ -229,6 +179,12 @@
   </si>
   <si>
     <t>[Gestión Hídrica El Soldado] Pozo El Melón N° 06 (PEM-06) Nodo</t>
+  </si>
+  <si>
+    <t>05/12/2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Superintendencia de recursos hidricos </t>
   </si>
   <si>
     <t xml:space="preserve">PEM-06
@@ -421,6 +377,9 @@
     <t>Leonardo Gonzalez</t>
   </si>
   <si>
+    <t xml:space="preserve">Mantenimiento preventivo </t>
+  </si>
+  <si>
     <t>[Gestión Hídrica El Soldado] Pozo Los Litres N° 03 (PLL-03) Nodo 168</t>
   </si>
   <si>
@@ -560,9 +519,37 @@
     <t xml:space="preserve">Se realizo inspección visual de cada punto para que no se encontrarán bandalizado o con algún problema. </t>
   </si>
   <si>
+    <t>[Gestión Hídrica El Soldado] Pozo El Melón N° 10 (PEM-10) Nodo A16</t>
+  </si>
+  <si>
     <t>Se da revisión al punto por que ese encontraba caído y dando datos erróneos la sonda. 
 Se deja sonda con agua ya que se encontraba sin agua.
 Válvula estaba abierta. Habían indicios qué el agua había corrido por el piso hacia el exterior.</t>
+  </si>
+  <si>
+    <t>Visita terreno</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AAES </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Galileo estación reelevadora </t>
+  </si>
+  <si>
+    <t>05/01/2026</t>
+  </si>
+  <si>
+    <t>Se acude al punto a verificar la condición y se anota lo que falta para la habilitación de éste.
+Batería acorde y peinado de cables</t>
+  </si>
+  <si>
+    <t>Gestiones</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Se coordina con Joanil Contreras para la entrega de perfil metálico para instalación de lector de velocidad RQ30.
+- Se hace entrega de documentación a Sr. Nicolas solicitado por Rodrigo López.
+- Se espero a don Diego Ramos para la verificación de instalación de los postes en los puntos PEM, pero no fue posible reunirnos, esta coordinado para hoy a las 10:00hrs apox.
+- Se rotula las herramientas acorde al color reactivo de este mes. </t>
   </si>
   <si>
     <t>Ángel Zamora</t>
@@ -713,6 +700,26 @@
   <si>
     <t>PH de entrada en planta Biodiversa zona 1 esta desconectado del equipo, por ende marca dato erroneo.
 En planta Biodiversa vdf ksb pantalla no enciende, voltimetro marca más de 500v puede que el equipo falle lo que provocaría perdida de lecturas modbus.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Migración Red Lora </t>
+  </si>
+  <si>
+    <t>[Global Tórtolas] Pozo BN7</t>
+  </si>
+  <si>
+    <t>Durante mañana tarde firmas de PT, se retiran equipos de Netaxion.
+Paula Riquelme nos hace entrega de antenas Lora.
+Tiempo restante para migrar BN7 a Lora Wan, se dejan con Paula 21 equipos de estos guardados en su oficina.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Uc300 </t>
+  </si>
+  <si>
+    <t>6445F15714530004</t>
+  </si>
+  <si>
+    <t>Punto queda transmitiendo y operativo</t>
   </si>
 </sst>
 </file>
@@ -1125,7 +1132,7 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="B2" t="s">
         <v>25</v>
@@ -1140,16 +1147,16 @@
         <v>28</v>
       </c>
       <c r="F2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G2" t="s">
         <v>29</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>30</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>31</v>
-      </c>
-      <c r="I2" t="s">
-        <v>32</v>
       </c>
       <c r="J2">
         <v>5</v>
@@ -1157,31 +1164,31 @@
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A3">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="B3" t="s">
-        <v>33</v>
+        <v>14</v>
       </c>
       <c r="C3" t="s">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="D3" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="E3" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
       <c r="F3" t="s">
         <v>18</v>
       </c>
       <c r="G3" t="s">
-        <v>36</v>
+        <v>19</v>
       </c>
       <c r="H3" t="s">
-        <v>37</v>
+        <v>20</v>
       </c>
       <c r="I3" t="s">
-        <v>38</v>
+        <v>21</v>
       </c>
       <c r="J3">
         <v>5</v>
@@ -1189,31 +1196,31 @@
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A4">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="B4" t="s">
-        <v>33</v>
+        <v>14</v>
       </c>
       <c r="C4" t="s">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="D4" t="s">
         <v>22</v>
       </c>
       <c r="E4" t="s">
-        <v>39</v>
+        <v>23</v>
       </c>
       <c r="F4" t="s">
         <v>18</v>
       </c>
       <c r="G4" t="s">
-        <v>36</v>
+        <v>19</v>
       </c>
       <c r="H4" t="s">
-        <v>37</v>
+        <v>20</v>
       </c>
       <c r="I4" t="s">
-        <v>40</v>
+        <v>24</v>
       </c>
       <c r="J4">
         <v>5</v>
@@ -1221,31 +1228,31 @@
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A5">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="B5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C5" t="s">
         <v>33</v>
       </c>
-      <c r="C5" t="s">
-        <v>41</v>
-      </c>
       <c r="D5" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="E5" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="F5" t="s">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="G5" t="s">
-        <v>44</v>
+        <v>29</v>
       </c>
       <c r="H5" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="I5" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="J5">
         <v>5</v>
@@ -1253,63 +1260,75 @@
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A6">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="B6" t="s">
-        <v>14</v>
+        <v>149</v>
       </c>
       <c r="C6" t="s">
-        <v>15</v>
+        <v>64</v>
       </c>
       <c r="D6" t="s">
-        <v>16</v>
+        <v>121</v>
       </c>
       <c r="E6" t="s">
-        <v>17</v>
+        <v>150</v>
       </c>
       <c r="F6" t="s">
-        <v>18</v>
+        <v>151</v>
       </c>
       <c r="G6" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="H6" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="I6" t="s">
-        <v>21</v>
+        <v>152</v>
       </c>
       <c r="J6">
         <v>5</v>
+      </c>
+      <c r="K6" t="s">
+        <v>153</v>
+      </c>
+      <c r="L6" t="s">
+        <v>154</v>
+      </c>
+      <c r="M6" t="s">
+        <v>155</v>
+      </c>
+      <c r="N6" t="s">
+        <v>156</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A7">
-        <v>321</v>
+        <v>325</v>
       </c>
       <c r="B7" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="C7" t="s">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="D7" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="E7" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="F7" t="s">
         <v>18</v>
       </c>
       <c r="G7" t="s">
-        <v>19</v>
+        <v>41</v>
       </c>
       <c r="H7" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="I7" t="s">
-        <v>24</v>
+        <v>42</v>
       </c>
       <c r="J7">
         <v>5</v>
@@ -1317,31 +1336,31 @@
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A8">
-        <v>322</v>
+        <v>326</v>
       </c>
       <c r="B8" t="s">
-        <v>47</v>
+        <v>14</v>
       </c>
       <c r="C8" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="D8" t="s">
-        <v>49</v>
+        <v>22</v>
       </c>
       <c r="E8" t="s">
-        <v>50</v>
+        <v>23</v>
       </c>
       <c r="F8" t="s">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="G8" t="s">
+        <v>41</v>
+      </c>
+      <c r="H8" t="s">
+        <v>20</v>
+      </c>
+      <c r="I8" t="s">
         <v>44</v>
-      </c>
-      <c r="H8" t="s">
-        <v>51</v>
-      </c>
-      <c r="I8" t="s">
-        <v>52</v>
       </c>
       <c r="J8">
         <v>5</v>
@@ -1349,78 +1368,90 @@
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A9">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="B9" t="s">
-        <v>152</v>
+        <v>14</v>
       </c>
       <c r="C9" t="s">
-        <v>76</v>
+        <v>43</v>
       </c>
       <c r="D9" t="s">
-        <v>132</v>
+        <v>22</v>
       </c>
       <c r="E9" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="F9" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="G9" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="H9" t="s">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="I9" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="J9">
         <v>5</v>
       </c>
       <c r="K9" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="L9" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="M9" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="N9" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A10">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="B10" t="s">
-        <v>33</v>
+        <v>14</v>
       </c>
       <c r="C10" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="D10" t="s">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="E10" t="s">
-        <v>54</v>
+        <v>157</v>
       </c>
       <c r="F10" t="s">
-        <v>18</v>
+        <v>158</v>
       </c>
       <c r="G10" t="s">
-        <v>55</v>
+        <v>41</v>
       </c>
       <c r="H10" t="s">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="I10" t="s">
-        <v>56</v>
+        <v>159</v>
       </c>
       <c r="J10">
         <v>5</v>
+      </c>
+      <c r="K10" t="s">
+        <v>164</v>
+      </c>
+      <c r="L10" t="s">
+        <v>165</v>
+      </c>
+      <c r="M10" t="s">
+        <v>166</v>
+      </c>
+      <c r="N10" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.2">
@@ -1431,189 +1462,177 @@
         <v>14</v>
       </c>
       <c r="C11" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="D11" t="s">
         <v>22</v>
       </c>
       <c r="E11" t="s">
-        <v>23</v>
+        <v>157</v>
       </c>
       <c r="F11" t="s">
-        <v>18</v>
+        <v>158</v>
       </c>
       <c r="G11" t="s">
-        <v>55</v>
+        <v>41</v>
       </c>
       <c r="H11" t="s">
         <v>20</v>
       </c>
       <c r="I11" t="s">
-        <v>58</v>
+        <v>159</v>
       </c>
       <c r="J11">
         <v>5</v>
+      </c>
+      <c r="K11" t="s">
+        <v>153</v>
+      </c>
+      <c r="L11" t="s">
+        <v>168</v>
+      </c>
+      <c r="M11" t="s">
+        <v>169</v>
+      </c>
+      <c r="N11" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A12">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="B12" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="C12" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="D12" t="s">
         <v>22</v>
       </c>
       <c r="E12" t="s">
-        <v>160</v>
+        <v>46</v>
       </c>
       <c r="F12" t="s">
-        <v>161</v>
+        <v>18</v>
       </c>
       <c r="G12" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="H12" t="s">
-        <v>20</v>
+        <v>48</v>
       </c>
       <c r="I12" t="s">
-        <v>162</v>
+        <v>49</v>
       </c>
       <c r="J12">
         <v>5</v>
-      </c>
-      <c r="K12" t="s">
-        <v>163</v>
-      </c>
-      <c r="L12" t="s">
-        <v>164</v>
-      </c>
-      <c r="M12" t="s">
-        <v>165</v>
-      </c>
-      <c r="N12" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A13">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="B13" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="C13" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="D13" t="s">
-        <v>22</v>
+        <v>50</v>
       </c>
       <c r="E13" t="s">
-        <v>160</v>
+        <v>51</v>
       </c>
       <c r="F13" t="s">
-        <v>161</v>
+        <v>18</v>
       </c>
       <c r="G13" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="H13" t="s">
-        <v>20</v>
+        <v>48</v>
       </c>
       <c r="I13" t="s">
-        <v>162</v>
+        <v>52</v>
       </c>
       <c r="J13">
         <v>5</v>
-      </c>
-      <c r="K13" t="s">
-        <v>167</v>
-      </c>
-      <c r="L13" t="s">
-        <v>168</v>
-      </c>
-      <c r="M13" t="s">
-        <v>169</v>
-      </c>
-      <c r="N13" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A14">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="B14" t="s">
-        <v>14</v>
+        <v>149</v>
       </c>
       <c r="C14" t="s">
-        <v>57</v>
+        <v>171</v>
       </c>
       <c r="D14" t="s">
         <v>22</v>
       </c>
       <c r="E14" t="s">
-        <v>160</v>
+        <v>172</v>
       </c>
       <c r="F14" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="G14" t="s">
-        <v>55</v>
+        <v>41</v>
       </c>
       <c r="H14" t="s">
-        <v>20</v>
+        <v>173</v>
       </c>
       <c r="I14" t="s">
+        <v>174</v>
+      </c>
+      <c r="J14">
+        <v>5</v>
+      </c>
+      <c r="K14" t="s">
+        <v>175</v>
+      </c>
+      <c r="L14" t="s">
+        <v>176</v>
+      </c>
+      <c r="M14" t="s">
+        <v>177</v>
+      </c>
+      <c r="N14" t="s">
         <v>162</v>
-      </c>
-      <c r="J14">
-        <v>5</v>
-      </c>
-      <c r="K14" t="s">
-        <v>156</v>
-      </c>
-      <c r="L14" t="s">
-        <v>171</v>
-      </c>
-      <c r="M14" t="s">
-        <v>172</v>
-      </c>
-      <c r="N14" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A15">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="B15" t="s">
-        <v>33</v>
+        <v>53</v>
       </c>
       <c r="C15" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="D15" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="E15" t="s">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="F15" t="s">
         <v>18</v>
       </c>
       <c r="G15" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="H15" t="s">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="I15" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="J15">
         <v>5</v>
@@ -1621,31 +1640,31 @@
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A16">
-        <v>327</v>
+        <v>334</v>
       </c>
       <c r="B16" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="C16" t="s">
+        <v>57</v>
+      </c>
+      <c r="D16" t="s">
+        <v>22</v>
+      </c>
+      <c r="E16" t="s">
+        <v>58</v>
+      </c>
+      <c r="F16" t="s">
+        <v>18</v>
+      </c>
+      <c r="G16" t="s">
         <v>59</v>
       </c>
-      <c r="D16" t="s">
-        <v>62</v>
-      </c>
-      <c r="E16" t="s">
-        <v>63</v>
-      </c>
-      <c r="F16" t="s">
-        <v>18</v>
-      </c>
-      <c r="G16" t="s">
-        <v>36</v>
-      </c>
       <c r="H16" t="s">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="I16" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="J16">
         <v>5</v>
@@ -1653,107 +1672,107 @@
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A17">
-        <v>329</v>
+        <v>336</v>
       </c>
       <c r="B17" t="s">
-        <v>152</v>
+        <v>53</v>
       </c>
       <c r="C17" t="s">
-        <v>174</v>
+        <v>61</v>
       </c>
       <c r="D17" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="E17" t="s">
-        <v>175</v>
+        <v>40</v>
       </c>
       <c r="F17" t="s">
-        <v>161</v>
+        <v>18</v>
       </c>
       <c r="G17" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="H17" t="s">
-        <v>176</v>
+        <v>30</v>
       </c>
       <c r="I17" t="s">
-        <v>177</v>
+        <v>63</v>
       </c>
       <c r="J17">
         <v>5</v>
-      </c>
-      <c r="K17" t="s">
-        <v>178</v>
-      </c>
-      <c r="L17" t="s">
-        <v>179</v>
-      </c>
-      <c r="M17" t="s">
-        <v>180</v>
-      </c>
-      <c r="N17" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A18">
-        <v>330</v>
+        <v>337</v>
       </c>
       <c r="B18" t="s">
-        <v>65</v>
+        <v>149</v>
       </c>
       <c r="C18" t="s">
-        <v>66</v>
+        <v>178</v>
       </c>
       <c r="D18" t="s">
-        <v>42</v>
+        <v>121</v>
       </c>
       <c r="E18" t="s">
-        <v>54</v>
+        <v>179</v>
       </c>
       <c r="F18" t="s">
-        <v>18</v>
+        <v>180</v>
       </c>
       <c r="G18" t="s">
-        <v>55</v>
+        <v>69</v>
       </c>
       <c r="H18" t="s">
-        <v>67</v>
+        <v>30</v>
       </c>
       <c r="I18" t="s">
-        <v>68</v>
+        <v>181</v>
       </c>
       <c r="J18">
         <v>5</v>
+      </c>
+      <c r="K18" t="s">
+        <v>175</v>
+      </c>
+      <c r="L18" t="s">
+        <v>162</v>
+      </c>
+      <c r="M18" t="s">
+        <v>162</v>
+      </c>
+      <c r="N18" t="s">
+        <v>162</v>
       </c>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A19">
-        <v>334</v>
+        <v>338</v>
       </c>
       <c r="B19" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="C19" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="D19" t="s">
         <v>22</v>
       </c>
       <c r="E19" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="F19" t="s">
         <v>18</v>
       </c>
       <c r="G19" t="s">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="H19" t="s">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="I19" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="J19">
         <v>5</v>
@@ -1761,31 +1780,31 @@
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A20">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="B20" t="s">
-        <v>65</v>
+        <v>25</v>
       </c>
       <c r="C20" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="D20" t="s">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="E20" t="s">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="F20" t="s">
         <v>18</v>
       </c>
       <c r="G20" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="H20" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="I20" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="J20">
         <v>5</v>
@@ -1793,75 +1812,63 @@
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A21">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B21" t="s">
-        <v>152</v>
+        <v>25</v>
       </c>
       <c r="C21" t="s">
-        <v>181</v>
+        <v>67</v>
       </c>
       <c r="D21" t="s">
-        <v>132</v>
+        <v>22</v>
       </c>
       <c r="E21" t="s">
-        <v>182</v>
+        <v>71</v>
       </c>
       <c r="F21" t="s">
-        <v>183</v>
+        <v>18</v>
       </c>
       <c r="G21" t="s">
-        <v>81</v>
+        <v>69</v>
       </c>
       <c r="H21" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="I21" t="s">
-        <v>184</v>
+        <v>72</v>
       </c>
       <c r="J21">
         <v>5</v>
-      </c>
-      <c r="K21" t="s">
-        <v>178</v>
-      </c>
-      <c r="L21" t="s">
-        <v>165</v>
-      </c>
-      <c r="M21" t="s">
-        <v>165</v>
-      </c>
-      <c r="N21" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A22">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="B22" t="s">
-        <v>33</v>
+        <v>53</v>
       </c>
       <c r="C22" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="D22" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="E22" t="s">
-        <v>77</v>
+        <v>40</v>
       </c>
       <c r="F22" t="s">
         <v>18</v>
       </c>
       <c r="G22" t="s">
+        <v>69</v>
+      </c>
+      <c r="H22" t="s">
+        <v>55</v>
+      </c>
+      <c r="I22" t="s">
         <v>74</v>
-      </c>
-      <c r="H22" t="s">
-        <v>37</v>
-      </c>
-      <c r="I22" t="s">
-        <v>78</v>
       </c>
       <c r="J22">
         <v>5</v>
@@ -1869,31 +1876,31 @@
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A23">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="B23" t="s">
-        <v>33</v>
+        <v>53</v>
       </c>
       <c r="C23" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="D23" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="E23" t="s">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="F23" t="s">
         <v>18</v>
       </c>
       <c r="G23" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="H23" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="I23" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="J23">
         <v>5</v>
@@ -1901,31 +1908,31 @@
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A24">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="B24" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="C24" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D24" t="s">
         <v>22</v>
       </c>
       <c r="E24" t="s">
-        <v>83</v>
+        <v>58</v>
       </c>
       <c r="F24" t="s">
         <v>18</v>
       </c>
       <c r="G24" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="H24" t="s">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="I24" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="J24">
         <v>5</v>
@@ -1933,31 +1940,31 @@
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A25">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="B25" t="s">
-        <v>65</v>
+        <v>25</v>
       </c>
       <c r="C25" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="D25" t="s">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="E25" t="s">
-        <v>54</v>
+        <v>81</v>
       </c>
       <c r="F25" t="s">
         <v>18</v>
       </c>
       <c r="G25" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="H25" t="s">
-        <v>67</v>
+        <v>48</v>
       </c>
       <c r="I25" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="J25">
         <v>5</v>
@@ -1965,31 +1972,31 @@
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A26">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="B26" t="s">
-        <v>65</v>
+        <v>83</v>
       </c>
       <c r="C26" t="s">
+        <v>84</v>
+      </c>
+      <c r="D26" t="s">
+        <v>85</v>
+      </c>
+      <c r="E26" t="s">
+        <v>86</v>
+      </c>
+      <c r="F26" t="s">
         <v>87</v>
-      </c>
-      <c r="D26" t="s">
-        <v>42</v>
-      </c>
-      <c r="E26" t="s">
-        <v>54</v>
-      </c>
-      <c r="F26" t="s">
-        <v>18</v>
       </c>
       <c r="G26" t="s">
         <v>88</v>
       </c>
       <c r="H26" t="s">
-        <v>45</v>
+        <v>89</v>
       </c>
       <c r="I26" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="J26">
         <v>5</v>
@@ -1997,31 +2004,31 @@
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A27">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="B27" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="C27" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D27" t="s">
-        <v>22</v>
+        <v>92</v>
       </c>
       <c r="E27" t="s">
-        <v>70</v>
+        <v>93</v>
       </c>
       <c r="F27" t="s">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="G27" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="H27" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="I27" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="J27">
         <v>5</v>
@@ -2029,16 +2036,16 @@
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A28">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="B28" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="C28" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D28" t="s">
-        <v>22</v>
+        <v>92</v>
       </c>
       <c r="E28" t="s">
         <v>93</v>
@@ -2047,13 +2054,13 @@
         <v>18</v>
       </c>
       <c r="G28" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="H28" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="I28" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J28">
         <v>5</v>
@@ -2061,31 +2068,31 @@
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A29">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="B29" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C29" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D29" t="s">
-        <v>97</v>
+        <v>22</v>
       </c>
       <c r="E29" t="s">
         <v>98</v>
       </c>
       <c r="F29" t="s">
+        <v>18</v>
+      </c>
+      <c r="G29" t="s">
+        <v>88</v>
+      </c>
+      <c r="H29" t="s">
         <v>99</v>
       </c>
-      <c r="G29" t="s">
+      <c r="I29" t="s">
         <v>100</v>
-      </c>
-      <c r="H29" t="s">
-        <v>101</v>
-      </c>
-      <c r="I29" t="s">
-        <v>102</v>
       </c>
       <c r="J29">
         <v>5</v>
@@ -2093,31 +2100,31 @@
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A30">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="B30" t="s">
-        <v>33</v>
+        <v>83</v>
       </c>
       <c r="C30" t="s">
+        <v>101</v>
+      </c>
+      <c r="D30" t="s">
+        <v>102</v>
+      </c>
+      <c r="E30" t="s">
         <v>103</v>
       </c>
-      <c r="D30" t="s">
+      <c r="F30" t="s">
+        <v>18</v>
+      </c>
+      <c r="G30" t="s">
+        <v>94</v>
+      </c>
+      <c r="H30" t="s">
         <v>104</v>
       </c>
-      <c r="E30" t="s">
+      <c r="I30" t="s">
         <v>105</v>
-      </c>
-      <c r="F30" t="s">
-        <v>29</v>
-      </c>
-      <c r="G30" t="s">
-        <v>106</v>
-      </c>
-      <c r="H30" t="s">
-        <v>45</v>
-      </c>
-      <c r="I30" t="s">
-        <v>107</v>
       </c>
       <c r="J30">
         <v>5</v>
@@ -2125,31 +2132,31 @@
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A31">
-        <v>345</v>
+        <v>349</v>
       </c>
       <c r="B31" t="s">
-        <v>33</v>
+        <v>53</v>
       </c>
       <c r="C31" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="D31" t="s">
-        <v>104</v>
+        <v>93</v>
       </c>
       <c r="E31" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F31" t="s">
         <v>18</v>
       </c>
       <c r="G31" t="s">
-        <v>106</v>
+        <v>94</v>
       </c>
       <c r="H31" t="s">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="I31" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="J31">
         <v>5</v>
@@ -2157,28 +2164,28 @@
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A32">
-        <v>347</v>
+        <v>351</v>
       </c>
       <c r="B32" t="s">
-        <v>108</v>
+        <v>96</v>
       </c>
       <c r="C32" t="s">
-        <v>34</v>
+        <v>97</v>
       </c>
       <c r="D32" t="s">
-        <v>22</v>
+        <v>109</v>
       </c>
       <c r="E32" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F32" t="s">
         <v>18</v>
       </c>
       <c r="G32" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="H32" t="s">
-        <v>110</v>
+        <v>99</v>
       </c>
       <c r="I32" t="s">
         <v>111</v>
@@ -2189,31 +2196,31 @@
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A33">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="B33" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C33" t="s">
+        <v>97</v>
+      </c>
+      <c r="D33" t="s">
+        <v>22</v>
+      </c>
+      <c r="E33" t="s">
         <v>112</v>
       </c>
-      <c r="D33" t="s">
+      <c r="F33" t="s">
+        <v>18</v>
+      </c>
+      <c r="G33" t="s">
+        <v>94</v>
+      </c>
+      <c r="H33" t="s">
+        <v>99</v>
+      </c>
+      <c r="I33" t="s">
         <v>113</v>
-      </c>
-      <c r="E33" t="s">
-        <v>114</v>
-      </c>
-      <c r="F33" t="s">
-        <v>18</v>
-      </c>
-      <c r="G33" t="s">
-        <v>106</v>
-      </c>
-      <c r="H33" t="s">
-        <v>115</v>
-      </c>
-      <c r="I33" t="s">
-        <v>116</v>
       </c>
       <c r="J33">
         <v>5</v>
@@ -2221,31 +2228,31 @@
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A34">
-        <v>349</v>
+        <v>353</v>
       </c>
       <c r="B34" t="s">
-        <v>65</v>
+        <v>96</v>
       </c>
       <c r="C34" t="s">
-        <v>117</v>
+        <v>97</v>
       </c>
       <c r="D34" t="s">
-        <v>105</v>
+        <v>22</v>
       </c>
       <c r="E34" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="F34" t="s">
         <v>18</v>
       </c>
       <c r="G34" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="H34" t="s">
-        <v>45</v>
+        <v>99</v>
       </c>
       <c r="I34" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="J34">
         <v>5</v>
@@ -2253,31 +2260,31 @@
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A35">
-        <v>351</v>
+        <v>355</v>
       </c>
       <c r="B35" t="s">
-        <v>108</v>
+        <v>96</v>
       </c>
       <c r="C35" t="s">
-        <v>34</v>
+        <v>97</v>
       </c>
       <c r="D35" t="s">
-        <v>120</v>
+        <v>109</v>
       </c>
       <c r="E35" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="F35" t="s">
         <v>18</v>
       </c>
       <c r="G35" t="s">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="H35" t="s">
-        <v>110</v>
+        <v>99</v>
       </c>
       <c r="I35" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="J35">
         <v>5</v>
@@ -2285,28 +2292,28 @@
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A36">
-        <v>351</v>
+        <v>356</v>
       </c>
       <c r="B36" t="s">
-        <v>108</v>
+        <v>53</v>
       </c>
       <c r="C36" t="s">
-        <v>34</v>
+        <v>120</v>
       </c>
       <c r="D36" t="s">
-        <v>22</v>
+        <v>121</v>
       </c>
       <c r="E36" t="s">
+        <v>122</v>
+      </c>
+      <c r="F36" t="s">
+        <v>18</v>
+      </c>
+      <c r="G36" t="s">
         <v>123</v>
       </c>
-      <c r="F36" t="s">
-        <v>18</v>
-      </c>
-      <c r="G36" t="s">
-        <v>106</v>
-      </c>
       <c r="H36" t="s">
-        <v>110</v>
+        <v>30</v>
       </c>
       <c r="I36" t="s">
         <v>124</v>
@@ -2317,16 +2324,16 @@
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A37">
-        <v>353</v>
+        <v>357</v>
       </c>
       <c r="B37" t="s">
-        <v>108</v>
+        <v>96</v>
       </c>
       <c r="C37" t="s">
-        <v>34</v>
+        <v>97</v>
       </c>
       <c r="D37" t="s">
-        <v>22</v>
+        <v>109</v>
       </c>
       <c r="E37" t="s">
         <v>125</v>
@@ -2338,7 +2345,7 @@
         <v>126</v>
       </c>
       <c r="H37" t="s">
-        <v>110</v>
+        <v>99</v>
       </c>
       <c r="I37" t="s">
         <v>127</v>
@@ -2349,31 +2356,31 @@
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A38">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="B38" t="s">
-        <v>108</v>
+        <v>96</v>
       </c>
       <c r="C38" t="s">
-        <v>34</v>
+        <v>97</v>
       </c>
       <c r="D38" t="s">
-        <v>120</v>
+        <v>22</v>
       </c>
       <c r="E38" t="s">
+        <v>114</v>
+      </c>
+      <c r="F38" t="s">
+        <v>18</v>
+      </c>
+      <c r="G38" t="s">
+        <v>126</v>
+      </c>
+      <c r="H38" t="s">
+        <v>99</v>
+      </c>
+      <c r="I38" t="s">
         <v>128</v>
-      </c>
-      <c r="F38" t="s">
-        <v>18</v>
-      </c>
-      <c r="G38" t="s">
-        <v>129</v>
-      </c>
-      <c r="H38" t="s">
-        <v>110</v>
-      </c>
-      <c r="I38" t="s">
-        <v>130</v>
       </c>
       <c r="J38">
         <v>5</v>
@@ -2381,31 +2388,31 @@
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A39">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="B39" t="s">
-        <v>65</v>
+        <v>96</v>
       </c>
       <c r="C39" t="s">
-        <v>131</v>
+        <v>97</v>
       </c>
       <c r="D39" t="s">
-        <v>132</v>
+        <v>109</v>
       </c>
       <c r="E39" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="F39" t="s">
         <v>18</v>
       </c>
       <c r="G39" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="H39" t="s">
-        <v>45</v>
+        <v>99</v>
       </c>
       <c r="I39" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="J39">
         <v>5</v>
@@ -2413,48 +2420,60 @@
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A40">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="B40" t="s">
-        <v>108</v>
+        <v>149</v>
       </c>
       <c r="C40" t="s">
-        <v>34</v>
+        <v>182</v>
       </c>
       <c r="D40" t="s">
-        <v>120</v>
+        <v>183</v>
       </c>
       <c r="E40" t="s">
-        <v>136</v>
+        <v>184</v>
       </c>
       <c r="F40" t="s">
-        <v>18</v>
+        <v>180</v>
       </c>
       <c r="G40" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="H40" t="s">
-        <v>110</v>
+        <v>185</v>
       </c>
       <c r="I40" t="s">
-        <v>138</v>
+        <v>186</v>
       </c>
       <c r="J40">
         <v>5</v>
+      </c>
+      <c r="K40" t="s">
+        <v>175</v>
+      </c>
+      <c r="L40" t="s">
+        <v>162</v>
+      </c>
+      <c r="M40" t="s">
+        <v>162</v>
+      </c>
+      <c r="N40" t="s">
+        <v>187</v>
       </c>
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A41">
-        <v>357</v>
+        <v>361</v>
       </c>
       <c r="B41" t="s">
-        <v>108</v>
+        <v>96</v>
       </c>
       <c r="C41" t="s">
-        <v>34</v>
+        <v>97</v>
       </c>
       <c r="D41" t="s">
-        <v>22</v>
+        <v>109</v>
       </c>
       <c r="E41" t="s">
         <v>125</v>
@@ -2463,13 +2482,13 @@
         <v>18</v>
       </c>
       <c r="G41" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="H41" t="s">
-        <v>110</v>
+        <v>99</v>
       </c>
       <c r="I41" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="J41">
         <v>5</v>
@@ -2477,31 +2496,31 @@
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A42">
-        <v>357</v>
+        <v>361</v>
       </c>
       <c r="B42" t="s">
-        <v>108</v>
+        <v>96</v>
       </c>
       <c r="C42" t="s">
-        <v>34</v>
+        <v>97</v>
       </c>
       <c r="D42" t="s">
-        <v>120</v>
+        <v>132</v>
       </c>
       <c r="E42" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="F42" t="s">
         <v>18</v>
       </c>
       <c r="G42" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="H42" t="s">
-        <v>110</v>
+        <v>99</v>
       </c>
       <c r="I42" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="J42">
         <v>5</v>
@@ -2509,28 +2528,28 @@
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A43">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="B43" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="C43" t="s">
+        <v>188</v>
+      </c>
+      <c r="D43" t="s">
+        <v>183</v>
+      </c>
+      <c r="E43" t="s">
+        <v>184</v>
+      </c>
+      <c r="F43" t="s">
+        <v>180</v>
+      </c>
+      <c r="G43" t="s">
+        <v>130</v>
+      </c>
+      <c r="H43" t="s">
         <v>185</v>
-      </c>
-      <c r="D43" t="s">
-        <v>186</v>
-      </c>
-      <c r="E43" t="s">
-        <v>187</v>
-      </c>
-      <c r="F43" t="s">
-        <v>183</v>
-      </c>
-      <c r="G43" t="s">
-        <v>141</v>
-      </c>
-      <c r="H43" t="s">
-        <v>188</v>
       </c>
       <c r="I43" t="s">
         <v>189</v>
@@ -2539,13 +2558,13 @@
         <v>5</v>
       </c>
       <c r="K43" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="L43" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="M43" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="N43" t="s">
         <v>190</v>
@@ -2553,31 +2572,31 @@
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A44">
-        <v>361</v>
+        <v>365</v>
       </c>
       <c r="B44" t="s">
-        <v>108</v>
+        <v>96</v>
       </c>
       <c r="C44" t="s">
-        <v>34</v>
+        <v>97</v>
       </c>
       <c r="D44" t="s">
-        <v>120</v>
+        <v>22</v>
       </c>
       <c r="E44" t="s">
+        <v>135</v>
+      </c>
+      <c r="F44" t="s">
+        <v>18</v>
+      </c>
+      <c r="G44" t="s">
         <v>136</v>
       </c>
-      <c r="F44" t="s">
-        <v>18</v>
-      </c>
-      <c r="G44" t="s">
-        <v>141</v>
-      </c>
       <c r="H44" t="s">
-        <v>110</v>
+        <v>99</v>
       </c>
       <c r="I44" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="J44">
         <v>5</v>
@@ -2585,31 +2604,31 @@
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A45">
-        <v>361</v>
+        <v>365</v>
       </c>
       <c r="B45" t="s">
-        <v>108</v>
+        <v>96</v>
       </c>
       <c r="C45" t="s">
-        <v>34</v>
+        <v>97</v>
       </c>
       <c r="D45" t="s">
-        <v>143</v>
+        <v>109</v>
       </c>
       <c r="E45" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="F45" t="s">
         <v>18</v>
       </c>
       <c r="G45" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="H45" t="s">
-        <v>110</v>
+        <v>99</v>
       </c>
       <c r="I45" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="J45">
         <v>5</v>
@@ -2617,107 +2636,107 @@
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A46">
-        <v>362</v>
+        <v>365</v>
       </c>
       <c r="B46" t="s">
-        <v>152</v>
+        <v>96</v>
       </c>
       <c r="C46" t="s">
-        <v>191</v>
+        <v>97</v>
       </c>
       <c r="D46" t="s">
-        <v>186</v>
+        <v>22</v>
       </c>
       <c r="E46" t="s">
-        <v>187</v>
+        <v>140</v>
       </c>
       <c r="F46" t="s">
-        <v>183</v>
+        <v>18</v>
       </c>
       <c r="G46" t="s">
+        <v>136</v>
+      </c>
+      <c r="H46" t="s">
+        <v>99</v>
+      </c>
+      <c r="I46" t="s">
         <v>141</v>
       </c>
-      <c r="H46" t="s">
-        <v>188</v>
-      </c>
-      <c r="I46" t="s">
-        <v>192</v>
-      </c>
       <c r="J46">
         <v>5</v>
-      </c>
-      <c r="K46" t="s">
-        <v>178</v>
-      </c>
-      <c r="L46" t="s">
-        <v>165</v>
-      </c>
-      <c r="M46" t="s">
-        <v>165</v>
-      </c>
-      <c r="N46" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A47">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="B47" t="s">
-        <v>108</v>
+        <v>149</v>
       </c>
       <c r="C47" t="s">
-        <v>34</v>
+        <v>191</v>
       </c>
       <c r="D47" t="s">
-        <v>22</v>
+        <v>121</v>
       </c>
       <c r="E47" t="s">
-        <v>146</v>
+        <v>192</v>
       </c>
       <c r="F47" t="s">
-        <v>18</v>
+        <v>180</v>
       </c>
       <c r="G47" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="H47" t="s">
-        <v>110</v>
+        <v>30</v>
       </c>
       <c r="I47" t="s">
-        <v>148</v>
+        <v>193</v>
       </c>
       <c r="J47">
         <v>5</v>
+      </c>
+      <c r="K47" t="s">
+        <v>175</v>
+      </c>
+      <c r="L47" t="s">
+        <v>194</v>
+      </c>
+      <c r="M47" t="s">
+        <v>195</v>
+      </c>
+      <c r="N47" t="s">
+        <v>196</v>
       </c>
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A48">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="B48" t="s">
-        <v>108</v>
+        <v>25</v>
       </c>
       <c r="C48" t="s">
-        <v>34</v>
+        <v>142</v>
       </c>
       <c r="D48" t="s">
-        <v>120</v>
+        <v>143</v>
       </c>
       <c r="E48" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="F48" t="s">
         <v>18</v>
       </c>
       <c r="G48" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="H48" t="s">
-        <v>110</v>
+        <v>48</v>
       </c>
       <c r="I48" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="J48">
         <v>5</v>
@@ -2725,31 +2744,31 @@
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A49">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="B49" t="s">
-        <v>108</v>
+        <v>25</v>
       </c>
       <c r="C49" t="s">
-        <v>34</v>
+        <v>142</v>
       </c>
       <c r="D49" t="s">
-        <v>22</v>
+        <v>50</v>
       </c>
       <c r="E49" t="s">
-        <v>39</v>
+        <v>147</v>
       </c>
       <c r="F49" t="s">
         <v>18</v>
       </c>
       <c r="G49" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="H49" t="s">
-        <v>110</v>
+        <v>48</v>
       </c>
       <c r="I49" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="J49">
         <v>5</v>

</xml_diff>